<commit_message>
Password-protect excel_templates sheet and workbook locks with "bildyx"
Sheet protection and workbook structure locking in generate_excel_templates.py
were previously password-less, so anyone could remove them with a single
click in Excel. Both now require TEMPLATE_PASSWORD ("bildyx").

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/apps/api/data/excel_templates/certifications.xlsx
+++ b/apps/api/data/excel_templates/certifications.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection lockStructure="1"/>
+  <workbookProtection workbookPassword="DB2D" lockStructure="1"/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
@@ -518,7 +518,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="1"/>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="1" password="DB2D"/>
   <autoFilter ref="A1:M1"/>
   <dataValidations count="4">
     <dataValidation sqref="F2:F1048576" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid value" error="Please select a value from the dropdown list." type="list">

</xml_diff>

<commit_message>
export excel via bdd
</commit_message>
<xml_diff>
--- a/apps/api/data/excel_templates/certifications.xlsx
+++ b/apps/api/data/excel_templates/certifications.xlsx
@@ -528,11 +528,6 @@
           <t>CER-000001</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>8kSec</t>
-        </is>
-      </c>
       <c r="D2" t="inlineStr">
         <is>
           <t>Demonstrates expertise in securing Android applications through vulnerability analysis, reverse engineering, and code review.</t>
@@ -550,12 +545,12 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Mobile Security Engineer, Penetration Tester, AppSec Analyst, Security Researcher, Android Developer</t>
+          <t>Mobile Security Engineer;Penetration Tester;AppSec Analyst;Security Researcher;Android Developer</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Advanced</t>
+          <t>ADVANCED</t>
         </is>
       </c>
     </row>
@@ -570,11 +565,6 @@
           <t>CER-000002</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>8kSec</t>
-        </is>
-      </c>
       <c r="D3" t="inlineStr">
         <is>
           <t>Focuses on in-depth Android internals, malware analysis, and exploit development for mobile platforms.</t>
@@ -592,12 +582,12 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Security Researcher, Reverse Engineer, Malware Analyst, Mobile Security Expert, Ethical Hacker</t>
+          <t>Security Researcher;Reverse Engineer;Malware Analyst;Mobile Security Expert;Ethical Hacker</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Advanced</t>
+          <t>ADVANCED</t>
         </is>
       </c>
     </row>
@@ -612,11 +602,6 @@
           <t>CER-000003</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>8kSec</t>
-        </is>
-      </c>
       <c r="D4" t="inlineStr">
         <is>
           <t>Focuses on iOS app security, reverse engineering, and mobile threat defense.</t>
@@ -634,12 +619,12 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Mobile Security Engineer, Penetration Tester, Security Researcher, App Developer, Threat Analyst</t>
+          <t>Mobile Security Engineer;Penetration Tester;Security Researcher;App Developer;Threat Analyst</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Advanced</t>
+          <t>ADVANCED</t>
         </is>
       </c>
     </row>
@@ -654,11 +639,6 @@
           <t>CER-000004</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>8kSec</t>
-        </is>
-      </c>
       <c r="D5" t="inlineStr">
         <is>
           <t>Specializes in iOS vulnerability research, exploitation, and patch analysis.</t>
@@ -676,12 +656,12 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Security Researcher, Exploit Developer, Mobile Analyst, Reverse Engineer, Bug Hunter</t>
+          <t>Security Researcher;Exploit Developer;Mobile Analyst;Reverse Engineer;Bug Hunter</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Advanced</t>
+          <t>ADVANCED</t>
         </is>
       </c>
     </row>
@@ -696,11 +676,6 @@
           <t>CER-000005</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>8kSec</t>
-        </is>
-      </c>
       <c r="D6" t="inlineStr">
         <is>
           <t>Focuses on securing Android and iOS mobile environments and applications.</t>
@@ -718,12 +693,12 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Mobile Security Engineer, App Developer, Penetration Tester, Threat Analyst, Security Consultant</t>
+          <t>Mobile Security Engineer;App Developer;Penetration Tester;Threat Analyst;Security Consultant</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Advanced</t>
+          <t>ADVANCED</t>
         </is>
       </c>
     </row>
@@ -738,11 +713,6 @@
           <t>CER-000006</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>8kSec</t>
-        </is>
-      </c>
       <c r="D7" t="inlineStr">
         <is>
           <t>Recognizes advanced expertise in mobile app exploitation, reverse engineering, and secure code review.</t>
@@ -760,12 +730,12 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Mobile Penetration Tester, Security Researcher, Reverse Engineer, Red Team Specialist, App Security Analyst</t>
+          <t>Mobile Penetration Tester;Security Researcher;Reverse Engineer;Red Team Specialist;App Security Analyst</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Expert</t>
+          <t>EXPERT</t>
         </is>
       </c>
     </row>
@@ -780,11 +750,6 @@
           <t>CER-000007</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>ACI Financial Markets Association</t>
-        </is>
-      </c>
       <c r="D8" t="inlineStr">
         <is>
           <t>Provides foundational knowledge of financial market operations, instruments, and trading practices. Emphasizes ethics, risk management, and market structure.</t>
@@ -802,12 +767,12 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Dealer, Trader Assistant, Risk Analyst, Treasury Assistant, Banking Analyst</t>
+          <t>Dealer;Trader Assistant;Risk Analyst;Treasury Assistant;Banking Analyst</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Beginner</t>
+          <t>BEGINNER</t>
         </is>
       </c>
     </row>
@@ -822,11 +787,6 @@
           <t>CER-000008</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>ACI Financial Markets Association</t>
-        </is>
-      </c>
       <c r="D9" t="inlineStr">
         <is>
           <t>Builds understanding of back-office operations in financial markets. Covers trade settlement, reconciliation, and risk control in banking environments.</t>
@@ -844,12 +804,12 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Operations Analyst, Settlement Officer, Risk Controller, Treasury Operations Specialist, Banking Officer</t>
+          <t>Operations Analyst;Settlement Officer;Risk Controller;Treasury Operations Specialist;Banking Officer</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Intermediate</t>
+          <t>INTERMEDIATE</t>
         </is>
       </c>
     </row>
@@ -864,11 +824,6 @@
           <t>CER-000009</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Adobe</t>
-        </is>
-      </c>
       <c r="D10" t="inlineStr">
         <is>
           <t>This certification focuses on the practical use of Adobe Advertising Cloud for demand-side platform (DSP) operations. It covers campaign management, audience targeting, and performance optimization in digital advertising.</t>
@@ -881,17 +836,17 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Adobe Advertising Cloud, DSP Tools</t>
+          <t>Adobe Advertising Cloud;DSP Tools</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Digital Advertising Specialist, Campaign Manager, Media Buyer, Digital Marketing Analyst, Programmatic Advertising Expert</t>
+          <t>Digital Advertising Specialist;Campaign Manager;Media Buyer;Digital Marketing Analyst;Programmatic Advertising Expert</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>Intermediate</t>
+          <t>INTERMEDIATE</t>
         </is>
       </c>
     </row>
@@ -906,11 +861,6 @@
           <t>CER-000010</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Adobe</t>
-        </is>
-      </c>
       <c r="D11" t="inlineStr">
         <is>
           <t>This certification emphasizes search advertising strategies and optimization within Adobe Advertising Cloud. It teaches users how to manage search campaigns, analyze performance, and improve ROI.</t>
@@ -923,17 +873,17 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Adobe Advertising Cloud, SEM Tools</t>
+          <t>Adobe Advertising Cloud;SEM Tools</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Search Engine Marketing (SEM) Specialist, Paid Search Analyst, Digital Advertising Manager, Campaign Analyst, PPC Specialist</t>
+          <t>Search Engine Marketing (SEM) Specialist;Paid Search Analyst;Digital Advertising Manager;Campaign Analyst;PPC Specialist</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Intermediate</t>
+          <t>INTERMEDIATE</t>
         </is>
       </c>
     </row>
@@ -948,11 +898,6 @@
           <t>CER-000011</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>Adobe</t>
-        </is>
-      </c>
       <c r="D12" t="inlineStr">
         <is>
           <t>The Analytics Architect Master certification is for advanced users of Adobe Analytics. It involves in-depth knowledge of data collection, configuration, and architecture to set up and manage analytics implementations.</t>
@@ -965,17 +910,17 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Adobe Analytics, Data Integration Tools</t>
+          <t>Adobe Analytics;Data Integration Tools</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Analytics Architect, Data Integration Specialist, Analytics Consultant, Digital Analyst, Marketing Data Manager</t>
+          <t>Analytics Architect;Data Integration Specialist;Analytics Consultant;Digital Analyst;Marketing Data Manager</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>Expert</t>
+          <t>EXPERT</t>
         </is>
       </c>
     </row>
@@ -990,11 +935,6 @@
           <t>CER-000012</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Adobe</t>
-        </is>
-      </c>
       <c r="D13" t="inlineStr">
         <is>
           <t>This expert-level certification focuses on leveraging Adobe Analytics for advanced business insights. It includes data analysis, report customization, and optimizing analytics for decision-making in a business context.</t>
@@ -1007,17 +947,17 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Adobe Analytics, Business Intelligence Tools</t>
+          <t>Adobe Analytics;Business Intelligence Tools</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Business Analyst, Marketing Analyst, Data Analyst, Digital Marketing Manager, Performance Analyst</t>
+          <t>Business Analyst;Marketing Analyst;Data Analyst;Digital Marketing Manager;Performance Analyst</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>Expert</t>
+          <t>EXPERT</t>
         </is>
       </c>
     </row>
@@ -1032,11 +972,6 @@
           <t>CER-000013</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Adobe</t>
-        </is>
-      </c>
       <c r="D14" t="inlineStr">
         <is>
           <t>This certification focuses on using Adobe Analytics for business insights and reporting. It includes key skills like setting up reports, creating segments, and analyzing traffic and user behavior for marketing optimization.</t>
@@ -1049,17 +984,17 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Adobe Analytics, Reporting Tools</t>
+          <t>Adobe Analytics;Reporting Tools</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>Business Analyst, Digital Marketing Analyst, Marketing Analyst, Data Specialist, Performance Marketing Manager</t>
+          <t>Business Analyst;Digital Marketing Analyst;Marketing Analyst;Data Specialist;Performance Marketing Manager</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>Intermediate</t>
+          <t>INTERMEDIATE</t>
         </is>
       </c>
     </row>
@@ -1074,11 +1009,6 @@
           <t>CER-000014</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>Adobe</t>
-        </is>
-      </c>
       <c r="D15" t="inlineStr">
         <is>
           <t>This certification focuses on the fundamentals of data analysis using Adobe Analytics. It covers data collection, report building, and basic interpretation of user data to help businesses make data-driven decisions.</t>
@@ -1091,17 +1021,17 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Adobe Analytics, Data Analysis Tools</t>
+          <t>Adobe Analytics;Data Analysis Tools</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>Data Analyst, Marketing Analyst, Business Intelligence Analyst, Digital Analyst, Web Analyst</t>
+          <t>Data Analyst;Marketing Analyst;Business Intelligence Analyst;Digital Analyst;Web Analyst</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>Intermediate</t>
+          <t>INTERMEDIATE</t>
         </is>
       </c>
     </row>
@@ -1116,11 +1046,6 @@
           <t>CER-000015</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>Adobe</t>
-        </is>
-      </c>
       <c r="D16" t="inlineStr">
         <is>
           <t>The Developer Expert certification covers advanced configuration and customization of Adobe Analytics, focusing on implementation, data collection, and API integrations. Ideal for those working on technical aspects of analytics platforms.</t>
@@ -1133,17 +1058,17 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Adobe Analytics, API Integration Tools</t>
+          <t>Adobe Analytics;API Integration Tools</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>Analytics Developer, Web Developer, Data Integration Specialist, Technical Consultant, Analytics Engineer</t>
+          <t>Analytics Developer;Web Developer;Data Integration Specialist;Technical Consultant;Analytics Engineer</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>Expert</t>
+          <t>EXPERT</t>
         </is>
       </c>
     </row>
@@ -1158,11 +1083,6 @@
           <t>CER-000016</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>Adobe</t>
-        </is>
-      </c>
       <c r="D17" t="inlineStr">
         <is>
           <t>This certification focuses on the practical aspects of setting up and customizing Adobe Analytics for tracking and data collection. It’s ideal for developers who implement and maintain analytics solutions.</t>
@@ -1175,17 +1095,17 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Adobe Analytics, Data Collection Tools</t>
+          <t>Adobe Analytics;Data Collection Tools</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>Web Developer, Analytics Developer, Data Integration Specialist, Digital Analyst, Front-End Developer</t>
+          <t>Web Developer;Analytics Developer;Data Integration Specialist;Digital Analyst;Front-End Developer</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>Intermediate</t>
+          <t>INTERMEDIATE</t>
         </is>
       </c>
     </row>
@@ -1200,11 +1120,6 @@
           <t>CER-000017</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>Adobe</t>
-        </is>
-      </c>
       <c r="D18" t="inlineStr">
         <is>
           <t>This expert-level certification focuses on advanced configurations and architectures in Adobe Audience Manager. It covers data management, audience segmentation, and integration of Adobe solutions to enhance audience targeting.</t>
@@ -1217,17 +1132,17 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Adobe Audience Manager, Data Management Platform</t>
+          <t>Adobe Audience Manager;Data Management Platform</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>Audience Manager Architect, Data Architect, Digital Marketing Consultant, Data Integration Specialist, Campaign Manager</t>
+          <t>Audience Manager Architect;Data Architect;Digital Marketing Consultant;Data Integration Specialist;Campaign Manager</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>Expert</t>
+          <t>EXPERT</t>
         </is>
       </c>
     </row>
@@ -1242,11 +1157,6 @@
           <t>CER-000018</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>Adobe</t>
-        </is>
-      </c>
       <c r="D19" t="inlineStr">
         <is>
           <t>The Business Practitioner Expert certification focuses on leveraging Adobe Audience Manager for data segmentation, customer insights, and campaign targeting. It emphasizes using data effectively to optimize customer engagement and marketing performance.</t>
@@ -1259,17 +1169,17 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Adobe Audience Manager, Customer Segmentation Tools</t>
+          <t>Adobe Audience Manager;Customer Segmentation Tools</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>Marketing Analyst, Digital Advertising Specialist, Data Analyst, Campaign Manager, Marketing Manager</t>
+          <t>Marketing Analyst;Digital Advertising Specialist;Data Analyst;Campaign Manager;Marketing Manager</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>Expert</t>
+          <t>EXPERT</t>
         </is>
       </c>
     </row>
@@ -1284,11 +1194,6 @@
           <t>CER-000019</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>Adobe</t>
-        </is>
-      </c>
       <c r="D20" t="inlineStr">
         <is>
           <t>This certification provides practical knowledge of Adobe Audience Manager for audience data analysis, segmentation, and marketing personalization. It’s ideal for professionals implementing targeted advertising strategies.</t>
@@ -1301,17 +1206,17 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Adobe Audience Manager, Audience Segmentation Tools</t>
+          <t>Adobe Audience Manager;Audience Segmentation Tools</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>Digital Marketer, Campaign Manager, Audience Analyst, Marketing Specialist, Performance Analyst</t>
+          <t>Digital Marketer;Campaign Manager;Audience Analyst;Marketing Specialist;Performance Analyst</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>Intermediate</t>
+          <t>INTERMEDIATE</t>
         </is>
       </c>
     </row>
@@ -1326,11 +1231,6 @@
           <t>CER-000020</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>Adobe</t>
-        </is>
-      </c>
       <c r="D21" t="inlineStr">
         <is>
           <t>This advanced certification focuses on the architecture and strategic implementation of Adobe Campaign Classic. It covers data integration, workflow design, and managing marketing automation at scale.</t>
@@ -1343,17 +1243,17 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Adobe Campaign Classic, Marketing Automation Tools</t>
+          <t>Adobe Campaign Classic;Marketing Automation Tools</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>Campaign Architect, Marketing Automation Specialist, Campaign Manager, Technical Marketing Consultant, Solution Architect</t>
+          <t>Campaign Architect;Marketing Automation Specialist;Campaign Manager;Technical Marketing Consultant;Solution Architect</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>Expert</t>
+          <t>EXPERT</t>
         </is>
       </c>
     </row>
@@ -1368,11 +1268,6 @@
           <t>CER-000021</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>Adobe</t>
-        </is>
-      </c>
       <c r="D22" t="inlineStr">
         <is>
           <t>This certification emphasizes the use of Adobe Campaign Classic for campaign management, customer journey mapping, and personalized marketing. It’s geared towards advanced users looking to optimize customer engagement strategies.</t>
@@ -1385,17 +1280,17 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Adobe Campaign Classic, Campaign Management Tools</t>
+          <t>Adobe Campaign Classic;Campaign Management Tools</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>Campaign Manager, Marketing Automation Specialist, Digital Campaign Lead, Email Marketing Manager, Marketing Operations Director</t>
+          <t>Campaign Manager;Marketing Automation Specialist;Digital Campaign Lead;Email Marketing Manager;Marketing Operations Director</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>Expert</t>
+          <t>EXPERT</t>
         </is>
       </c>
     </row>
@@ -1410,11 +1305,6 @@
           <t>CER-000022</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>Adobe</t>
-        </is>
-      </c>
       <c r="D23" t="inlineStr">
         <is>
           <t>This certification focuses on using Adobe Campaign Classic for effective campaign execution, reporting, and analytics. It teaches users how to set up and run targeted email campaigns and measure marketing success.</t>
@@ -1427,17 +1317,17 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Adobe Campaign Classic, Email Campaign Tools</t>
+          <t>Adobe Campaign Classic;Email Campaign Tools</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>Campaign Specialist, Email Marketing Manager, Digital Marketing Coordinator, CRM Specialist, Campaign Analyst</t>
+          <t>Campaign Specialist;Email Marketing Manager;Digital Marketing Coordinator;CRM Specialist;Campaign Analyst</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>Intermediate</t>
+          <t>INTERMEDIATE</t>
         </is>
       </c>
     </row>
@@ -1452,11 +1342,6 @@
           <t>CER-000023</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>Adobe</t>
-        </is>
-      </c>
       <c r="D24" t="inlineStr">
         <is>
           <t>The Developer Expert certification covers advanced skills in developing and customizing Adobe Campaign Classic, including integrating data sources, automation, and API-driven workflows.</t>
@@ -1469,17 +1354,17 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Adobe Campaign Classic, API Integration, Workflow Automation</t>
+          <t>Adobe Campaign Classic;API Integration;Workflow Automation</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>Campaign Developer, Marketing Automation Developer, Data Integration Specialist, Technical Consultant, API Developer</t>
+          <t>Campaign Developer;Marketing Automation Developer;Data Integration Specialist;Technical Consultant;API Developer</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>Expert</t>
+          <t>EXPERT</t>
         </is>
       </c>
     </row>
@@ -1494,11 +1379,6 @@
           <t>CER-000024</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>Adobe</t>
-        </is>
-      </c>
       <c r="D25" t="inlineStr">
         <is>
           <t>This certification focuses on the practical skills required to develop and customize Adobe Campaign Classic. It includes tasks like creating custom workflows, data imports, and client-specific integrations.</t>
@@ -1511,17 +1391,17 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Adobe Campaign Classic, Data Import Tools</t>
+          <t>Adobe Campaign Classic;Data Import Tools</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>Campaign Developer, Marketing Automation Developer, CRM Developer, Data Integration Developer, Email Developer</t>
+          <t>Campaign Developer;Marketing Automation Developer;CRM Developer;Data Integration Developer;Email Developer</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>Intermediate</t>
+          <t>INTERMEDIATE</t>
         </is>
       </c>
     </row>
@@ -1536,11 +1416,6 @@
           <t>CER-000025</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>Adobe</t>
-        </is>
-      </c>
       <c r="D26" t="inlineStr">
         <is>
           <t>Validates proficiency in designing, implementing, and troubleshooting marketing campaigns using Adobe Campaign.</t>
@@ -1558,12 +1433,12 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>Marketing Automation Developer, CRM Engineer, Email Marketing Specialist, Campaign Developer, Marketing Technologist</t>
+          <t>Marketing Automation Developer;CRM Engineer;Email Marketing Specialist;Campaign Developer;Marketing Technologist</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>Intermediate</t>
+          <t>INTERMEDIATE</t>
         </is>
       </c>
     </row>
@@ -1578,11 +1453,6 @@
           <t>CER-000026</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>Adobe</t>
-        </is>
-      </c>
       <c r="D27" t="inlineStr">
         <is>
           <t>This expert-level certification dives deep into Adobe Campaign's development environment. It focuses on advanced development tasks such as custom workflows, system integration, and building tailored marketing solutions for large-scale campaigns.</t>
@@ -1595,17 +1465,17 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Adobe Campaign, Custom Workflow Tools</t>
+          <t>Adobe Campaign;Custom Workflow Tools</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>Marketing Automation Developer, CRM Specialist, Campaign Engineer, Solution Developer, Technical Consultant</t>
+          <t>Marketing Automation Developer;CRM Specialist;Campaign Engineer;Solution Developer;Technical Consultant</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>Expert</t>
+          <t>EXPERT</t>
         </is>
       </c>
     </row>
@@ -1620,11 +1490,6 @@
           <t>CER-000027</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>Adobe</t>
-        </is>
-      </c>
       <c r="D28" t="inlineStr">
         <is>
           <t>This certification targets professionals using Adobe Campaign Standard for building and executing cross-channel campaigns. It focuses on optimizing customer engagement through automation, segmentation, and campaign performance analysis.</t>
@@ -1637,17 +1502,17 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Adobe Campaign Standard, Cross-Channel Marketing</t>
+          <t>Adobe Campaign Standard;Cross-Channel Marketing</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>Campaign Specialist, Marketing Operations Expert, Email Marketing Manager, Digital Campaign Specialist, Marketing Automation Consultant</t>
+          <t>Campaign Specialist;Marketing Operations Expert;Email Marketing Manager;Digital Campaign Specialist;Marketing Automation Consultant</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>Expert</t>
+          <t>EXPERT</t>
         </is>
       </c>
     </row>
@@ -1662,11 +1527,6 @@
           <t>CER-000028</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>Adobe</t>
-        </is>
-      </c>
       <c r="D29" t="inlineStr">
         <is>
           <t>This certification is designed for professionals who use Adobe Captivate to create interactive eLearning content. It covers advanced features like responsive design, multimedia integration, and mobile compatibility.</t>
@@ -1679,17 +1539,17 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Adobe Captivate, eLearning Tools</t>
+          <t>Adobe Captivate;eLearning Tools</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>eLearning Developer, Instructional Designer, Content Developer, Training Specialist, eLearning Specialist</t>
+          <t>eLearning Developer;Instructional Designer;Content Developer;Training Specialist;eLearning Specialist</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>Advanced</t>
+          <t>ADVANCED</t>
         </is>
       </c>
     </row>
@@ -1704,11 +1564,6 @@
           <t>CER-000029</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>Adobe</t>
-        </is>
-      </c>
       <c r="D30" t="inlineStr">
         <is>
           <t>Demonstrates understanding of Adobe Analytics Processing Rules to manipulate and enhance data collection for reporting accuracy.</t>
@@ -1726,12 +1581,12 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>Data Analyst, Digital Analytics Specialist, Marketing Technologist, Web Analyst, Tagging Engineer</t>
+          <t>Data Analyst;Digital Analytics Specialist;Marketing Technologist;Web Analyst;Tagging Engineer</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>Intermediate</t>
+          <t>INTERMEDIATE</t>
         </is>
       </c>
     </row>
@@ -1746,11 +1601,6 @@
           <t>CER-000030</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>Adobe</t>
-        </is>
-      </c>
       <c r="D31" t="inlineStr">
         <is>
           <t>Certifies ability to translate business needs into AEM solutions, optimize workflows, and manage digital assets effectively.</t>
@@ -1768,12 +1618,12 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>Digital Strategist, AEM Consultant, Project Manager, Business Analyst, CMS Administrator</t>
+          <t>Digital Strategist;AEM Consultant;Project Manager;Business Analyst;CMS Administrator</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>Advanced</t>
+          <t>ADVANCED</t>
         </is>
       </c>
     </row>
@@ -1788,11 +1638,6 @@
           <t>CER-000031</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>Adobe</t>
-        </is>
-      </c>
       <c r="D32" t="inlineStr">
         <is>
           <t>Focuses on developing, extending, and integrating AEM Assets to manage and deliver digital content efficiently.</t>
@@ -1810,12 +1655,12 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>AEM Developer, Web Engineer, CMS Developer, Integration Specialist, Front-End Developer</t>
+          <t>AEM Developer;Web Engineer;CMS Developer;Integration Specialist;Front-End Developer</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>Intermediate</t>
+          <t>INTERMEDIATE</t>
         </is>
       </c>
     </row>
@@ -1830,11 +1675,6 @@
           <t>CER-000032</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>Adobe</t>
-        </is>
-      </c>
       <c r="D33" t="inlineStr">
         <is>
           <t>Validates expertise in automating, deploying, and maintaining Adobe Experience Manager (AEM) environments through CI/CD, performance tuning, and infrastructure management.</t>
@@ -1852,12 +1692,12 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>DevOps Engineer, AEM Administrator, Cloud Engineer, Systems Integrator, Site Reliability Engineer</t>
+          <t>DevOps Engineer;AEM Administrator;Cloud Engineer;Systems Integrator;Site Reliability Engineer</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>Advanced</t>
+          <t>ADVANCED</t>
         </is>
       </c>
     </row>
@@ -1872,11 +1712,6 @@
           <t>CER-000033</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>Adobe</t>
-        </is>
-      </c>
       <c r="D34" t="inlineStr">
         <is>
           <t>Demonstrates proficiency in creating eLearning modules, interactive simulations, and assessments using Adobe Captivate 5.5.</t>
@@ -1894,12 +1729,12 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>eLearning Developer, Instructional Designer, Training Specialist, Multimedia Producer, Education Technologist</t>
+          <t>eLearning Developer;Instructional Designer;Training Specialist;Multimedia Producer;Education Technologist</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>Intermediate</t>
+          <t>INTERMEDIATE</t>
         </is>
       </c>
     </row>
@@ -1914,11 +1749,6 @@
           <t>CER-000034</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>Adobe</t>
-        </is>
-      </c>
       <c r="D35" t="inlineStr">
         <is>
           <t>Focuses on integrating Captivate with Adobe eLearning Suite tools for developing and managing interactive online training.</t>
@@ -1936,12 +1766,12 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>Instructional Designer, Learning Consultant, eLearning Developer, LMS Specialist, Multimedia Designer</t>
+          <t>Instructional Designer;Learning Consultant;eLearning Developer;LMS Specialist;Multimedia Designer</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>Advanced</t>
+          <t>ADVANCED</t>
         </is>
       </c>
     </row>
@@ -1956,11 +1786,6 @@
           <t>CER-000035</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>Adobe</t>
-        </is>
-      </c>
       <c r="D36" t="inlineStr">
         <is>
           <t>Validates the ability to develop, deploy, and maintain dynamic web applications using Adobe ColdFusion 9.</t>
@@ -1978,12 +1803,12 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>Web Developer, Application Developer, Software Engineer, Backend Developer, Systems Programmer</t>
+          <t>Web Developer;Application Developer;Software Engineer;Backend Developer;Systems Programmer</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>Intermediate</t>
+          <t>INTERMEDIATE</t>
         </is>
       </c>
     </row>
@@ -1998,11 +1823,6 @@
           <t>CER-000036</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>Adobe</t>
-        </is>
-      </c>
       <c r="D37" t="inlineStr">
         <is>
           <t>Recognizes proficiency in configuring, customizing, and managing AEM 6 for digital content delivery and web experience management.</t>
@@ -2020,12 +1840,12 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>AEM Developer, CMS Engineer, Web Application Developer, Technical Consultant, Solutions Architect</t>
+          <t>AEM Developer;CMS Engineer;Web Application Developer;Technical Consultant;Solutions Architect</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>Advanced</t>
+          <t>ADVANCED</t>
         </is>
       </c>
     </row>
@@ -2040,11 +1860,6 @@
           <t>CER-000037</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>Adobe</t>
-        </is>
-      </c>
       <c r="D38" t="inlineStr">
         <is>
           <t>Certifies ability to develop rich internet applications (RIAs) using Adobe Flex 4.5 and ActionScript.</t>
@@ -2062,12 +1877,12 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>Front-End Developer, UI Engineer, Flash/Flex Developer, Software Engineer, Web Application Developer</t>
+          <t>Front-End Developer;UI Engineer;Flash/Flex Developer;Software Engineer;Web Application Developer</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>Intermediate</t>
+          <t>INTERMEDIATE</t>
         </is>
       </c>
     </row>
@@ -2082,11 +1897,6 @@
           <t>CER-000038</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>Adobe</t>
-        </is>
-      </c>
       <c r="D39" t="inlineStr">
         <is>
           <t>Validates proficiency in creating professional print and digital layouts, styles, and templates using Adobe InDesign.</t>
@@ -2104,12 +1914,12 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>Graphic Designer, Layout Artist, Publishing Specialist, Print Designer, Marketing Designer</t>
+          <t>Graphic Designer;Layout Artist;Publishing Specialist;Print Designer;Marketing Designer</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>Intermediate</t>
+          <t>INTERMEDIATE</t>
         </is>
       </c>
     </row>
@@ -2124,11 +1934,6 @@
           <t>CER-000039</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>Adobe</t>
-        </is>
-      </c>
       <c r="D40" t="inlineStr">
         <is>
           <t>Certifies expertise in image editing, retouching, and digital compositing using Adobe Photoshop.</t>
@@ -2146,12 +1951,12 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>Graphic Designer, Photo Editor, Digital Artist, Creative Specialist, Visual Designer</t>
+          <t>Graphic Designer;Photo Editor;Digital Artist;Creative Specialist;Visual Designer</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>Intermediate</t>
+          <t>INTERMEDIATE</t>
         </is>
       </c>
     </row>
@@ -2166,11 +1971,6 @@
           <t>CER-000040</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>Adobe</t>
-        </is>
-      </c>
       <c r="D41" t="inlineStr">
         <is>
           <t>Recognizes mastery across multiple Adobe Creative Cloud applications, demonstrating comprehensive creative workflow proficiency.</t>
@@ -2188,12 +1988,12 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>Senior Designer, Art Director, Creative Lead, Digital Media Specialist, Visual Communication Expert</t>
+          <t>Senior Designer;Art Director;Creative Lead;Digital Media Specialist;Visual Communication Expert</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>Expert</t>
+          <t>EXPERT</t>
         </is>
       </c>
     </row>
@@ -2208,11 +2008,6 @@
           <t>CER-000041</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>Adobe</t>
-        </is>
-      </c>
       <c r="D42" t="inlineStr">
         <is>
           <t>Focuses on designing and implementing scalable Adobe Commerce (Magento) architectures integrating business logic, APIs, and custom modules.</t>
@@ -2230,12 +2025,12 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>Commerce Architect, Solutions Architect, Magento Developer, eCommerce Consultant, Technical Lead</t>
+          <t>Commerce Architect;Solutions Architect;Magento Developer;eCommerce Consultant;Technical Lead</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>Expert</t>
+          <t>EXPERT</t>
         </is>
       </c>
     </row>
@@ -2250,11 +2045,6 @@
           <t>CER-000042</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>Adobe</t>
-        </is>
-      </c>
       <c r="D43" t="inlineStr">
         <is>
           <t>Demonstrates foundational skills in vector illustration, logo design, and layout creation using Adobe Illustrator.</t>
@@ -2272,12 +2062,12 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>Graphic Designer, Illustrator, Branding Specialist, Visual Designer, Print Artist</t>
+          <t>Graphic Designer;Illustrator;Branding Specialist;Visual Designer;Print Artist</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>Intermediate</t>
+          <t>INTERMEDIATE</t>
         </is>
       </c>
     </row>
@@ -2292,11 +2082,6 @@
           <t>CER-000043</t>
         </is>
       </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>Adobe</t>
-        </is>
-      </c>
       <c r="D44" t="inlineStr">
         <is>
           <t>Recognizes basic proficiency in image editing, correction, and compositing for print and web media.</t>
@@ -2314,12 +2099,12 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>Junior Graphic Designer, Photo Editor, Digital Imaging Assistant, Content Creator, Visual Artist</t>
+          <t>Junior Graphic Designer;Photo Editor;Digital Imaging Assistant;Content Creator;Visual Artist</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>Intermediate</t>
+          <t>INTERMEDIATE</t>
         </is>
       </c>
     </row>
@@ -2334,11 +2119,6 @@
           <t>CER-000044</t>
         </is>
       </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>Adobe</t>
-        </is>
-      </c>
       <c r="D45" t="inlineStr">
         <is>
           <t>Validates ability to edit and produce professional-quality videos using Adobe Premiere Pro.</t>
@@ -2356,12 +2136,12 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>Video Editor, Content Producer, Media Specialist, Film Editor, Multimedia Editor</t>
+          <t>Video Editor;Content Producer;Media Specialist;Film Editor;Multimedia Editor</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>Intermediate</t>
+          <t>INTERMEDIATE</t>
         </is>
       </c>
     </row>
@@ -2376,11 +2156,6 @@
           <t>CER-000045</t>
         </is>
       </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>Adobe</t>
-        </is>
-      </c>
       <c r="D46" t="inlineStr">
         <is>
           <t>Demonstrates skill in creating cohesive video projects using Premiere Pro and After Effects workflows.</t>
@@ -2398,12 +2173,12 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>Video Designer, Multimedia Producer, Video Editor, Content Creator, Post-Production Assistant</t>
+          <t>Video Designer;Multimedia Producer;Video Editor;Content Creator;Post-Production Assistant</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>Intermediate</t>
+          <t>INTERMEDIATE</t>
         </is>
       </c>
     </row>
@@ -2418,11 +2193,6 @@
           <t>CER-000046</t>
         </is>
       </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>Adobe</t>
-        </is>
-      </c>
       <c r="D47" t="inlineStr">
         <is>
           <t>Certifies understanding of core design principles using Photoshop and Illustrator for digital and print media.</t>
@@ -2440,12 +2210,12 @@
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>Graphic Designer, Creative Assistant, Marketing Designer, Visual Content Creator, Junior Art Director</t>
+          <t>Graphic Designer;Creative Assistant;Marketing Designer;Visual Content Creator;Junior Art Director</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>Intermediate</t>
+          <t>INTERMEDIATE</t>
         </is>
       </c>
     </row>
@@ -2460,11 +2230,6 @@
           <t>CER-000047</t>
         </is>
       </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>Adobe</t>
-        </is>
-      </c>
       <c r="D48" t="inlineStr">
         <is>
           <t>Focuses on designing and publishing responsive websites using Adobe Dreamweaver and related web tools.</t>
@@ -2482,12 +2247,12 @@
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>Web Designer, Front-End Developer, UI Designer, Digital Media Specialist, Web Content Manager</t>
+          <t>Web Designer;Front-End Developer;UI Designer;Digital Media Specialist;Web Content Manager</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>Intermediate</t>
+          <t>INTERMEDIATE</t>
         </is>
       </c>
     </row>
@@ -2502,11 +2267,6 @@
           <t>CER-000048</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>Adobe</t>
-        </is>
-      </c>
       <c r="D49" t="inlineStr">
         <is>
           <t>This certification focuses on advanced skills in using Adobe ColdFusion for building dynamic websites and web applications. It includes topics such as data integration, security features, and advanced programming techniques.</t>
@@ -2519,17 +2279,17 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>Adobe ColdFusion, Web Development Tools</t>
+          <t>Adobe ColdFusion;Web Development Tools</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>Web Developer, ColdFusion Developer, Application Developer, Backend Developer, Full-Stack Developer</t>
+          <t>Web Developer;ColdFusion Developer;Application Developer;Backend Developer;Full-Stack Developer</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>Advanced</t>
+          <t>ADVANCED</t>
         </is>
       </c>
     </row>
@@ -2544,11 +2304,6 @@
           <t>CER-000049</t>
         </is>
       </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>Adobe</t>
-        </is>
-      </c>
       <c r="D50" t="inlineStr">
         <is>
           <t>This expert-level certification focuses on building and scaling Adobe Commerce (Magento) architectures. It covers integration, customizations, and optimizing eCommerce systems for enterprise-level businesses.</t>
@@ -2561,17 +2316,17 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>Adobe Commerce (Magento), eCommerce Platforms</t>
+          <t>Adobe Commerce (Magento);eCommerce Platforms</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>eCommerce Architect, Solution Architect, Systems Integrator, Magento Consultant, Enterprise Architect</t>
+          <t>eCommerce Architect;Solution Architect;Systems Integrator;Magento Consultant;Enterprise Architect</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>Expert</t>
+          <t>EXPERT</t>
         </is>
       </c>
     </row>
@@ -2586,11 +2341,6 @@
           <t>CER-000050</t>
         </is>
       </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>Adobe</t>
-        </is>
-      </c>
       <c r="D51" t="inlineStr">
         <is>
           <t>This certification focuses on mastering Adobe Commerce for business strategy. It covers advanced knowledge of eCommerce platform management, including marketing, customer experience, and product management strategies.</t>
@@ -2603,17 +2353,17 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>Adobe Commerce (Magento), Business Strategy Tools</t>
+          <t>Adobe Commerce (Magento);Business Strategy Tools</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>eCommerce Manager, Business Analyst, Digital Marketing Manager, Marketing Director, Product Manager</t>
+          <t>eCommerce Manager;Business Analyst;Digital Marketing Manager;Marketing Director;Product Manager</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>Expert</t>
+          <t>EXPERT</t>
         </is>
       </c>
     </row>
@@ -2628,11 +2378,6 @@
           <t>CER-000051</t>
         </is>
       </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>Adobe</t>
-        </is>
-      </c>
       <c r="D52" t="inlineStr">
         <is>
           <t>This certification is for professionals looking to deepen their understanding of Adobe Commerce. It covers topics like product catalog management, payment systems, and customer experience optimization.</t>
@@ -2645,17 +2390,17 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>Adobe Commerce (Magento), Product Management Tools</t>
+          <t>Adobe Commerce (Magento);Product Management Tools</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>eCommerce Specialist, Business Analyst, Marketing Specialist, Digital Commerce Manager, Product Owner</t>
+          <t>eCommerce Specialist;Business Analyst;Marketing Specialist;Digital Commerce Manager;Product Owner</t>
         </is>
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>Advanced</t>
+          <t>ADVANCED</t>
         </is>
       </c>
     </row>
@@ -2670,11 +2415,6 @@
           <t>CER-000052</t>
         </is>
       </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>Adobe</t>
-        </is>
-      </c>
       <c r="D53" t="inlineStr">
         <is>
           <t>Focuses on developing and deploying cloud-based Adobe Commerce solutions. Covers cloud architecture, integration, CI/CD workflows, and performance tuning for scalable e-commerce environments.</t>
@@ -2692,12 +2432,12 @@
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>Cloud E-commerce Developer, Adobe Commerce Architect, DevOps Engineer, Solutions Developer, Technical Consultant</t>
+          <t>Cloud E-commerce Developer;Adobe Commerce Architect;DevOps Engineer;Solutions Developer;Technical Consultant</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>Advanced</t>
+          <t>ADVANCED</t>
         </is>
       </c>
     </row>
@@ -2712,11 +2452,6 @@
           <t>CER-000053</t>
         </is>
       </c>
-      <c r="C54" t="inlineStr">
-        <is>
-          <t>Adobe</t>
-        </is>
-      </c>
       <c r="D54" t="inlineStr">
         <is>
           <t>Designed for developers with foundational knowledge, this certification tests practical skills in Adobe Commerce setup, basic customization, and extension development. It ensures developers can implement standard commerce solutions efficiently.</t>
@@ -2734,12 +2469,12 @@
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>Magento Developer, Frontend Developer, Web Developer, Junior E-commerce Developer, Technical Support Engineer</t>
+          <t>Magento Developer;Frontend Developer;Web Developer;Junior E-commerce Developer;Technical Support Engineer</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>Intermediate</t>
+          <t>INTERMEDIATE</t>
         </is>
       </c>
     </row>
@@ -2754,11 +2489,6 @@
           <t>CER-000054</t>
         </is>
       </c>
-      <c r="C55" t="inlineStr">
-        <is>
-          <t>Adobe</t>
-        </is>
-      </c>
       <c r="D55" t="inlineStr">
         <is>
           <t>This certification validates advanced skills in Adobe Commerce development, including complex architecture, custom module development, and performance optimization. Professionals demonstrate deep expertise in designing scalable e-commerce solutions.</t>
@@ -2776,12 +2506,12 @@
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>Senior Magento Developer, E-commerce Solutions Architect, Adobe Commerce Consultant, Technical Lead, Web Application Developer</t>
+          <t>Senior Magento Developer;E-commerce Solutions Architect;Adobe Commerce Consultant;Technical Lead;Web Application Developer</t>
         </is>
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>Expert</t>
+          <t>EXPERT</t>
         </is>
       </c>
     </row>
@@ -2796,11 +2526,6 @@
           <t>CER-000055</t>
         </is>
       </c>
-      <c r="C56" t="inlineStr">
-        <is>
-          <t>Adobe</t>
-        </is>
-      </c>
       <c r="D56" t="inlineStr">
         <is>
           <t>This advanced certification is for developers working with Adobe Commerce (Magento). It covers the full scope of development, including customization, plugin development, and system integration.</t>
@@ -2813,17 +2538,17 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>Adobe Commerce (Magento), Development Tools</t>
+          <t>Adobe Commerce (Magento);Development Tools</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>Magento Developer, eCommerce Developer, Full-Stack Developer, Backend Developer, Solution Developer</t>
+          <t>Magento Developer;eCommerce Developer;Full-Stack Developer;Backend Developer;Solution Developer</t>
         </is>
       </c>
       <c r="J56" t="inlineStr">
         <is>
-          <t>Expert</t>
+          <t>EXPERT</t>
         </is>
       </c>
     </row>
@@ -2838,11 +2563,6 @@
           <t>CER-000056</t>
         </is>
       </c>
-      <c r="C57" t="inlineStr">
-        <is>
-          <t>Adobe</t>
-        </is>
-      </c>
       <c r="D57" t="inlineStr">
         <is>
           <t>The Professional-level certification focuses on essential development skills for Adobe Commerce. It includes topics like theme customization, module development, and database management.</t>
@@ -2855,17 +2575,17 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>Adobe Commerce (Magento), Web Development Tools</t>
+          <t>Adobe Commerce (Magento);Web Development Tools</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>Magento Developer, eCommerce Developer, Web Developer, Full-Stack Developer, PHP Developer</t>
+          <t>Magento Developer;eCommerce Developer;Web Developer;Full-Stack Developer;PHP Developer</t>
         </is>
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>Advanced</t>
+          <t>ADVANCED</t>
         </is>
       </c>
     </row>
@@ -2880,11 +2600,6 @@
           <t>CER-000057</t>
         </is>
       </c>
-      <c r="C58" t="inlineStr">
-        <is>
-          <t>Adobe</t>
-        </is>
-      </c>
       <c r="D58" t="inlineStr">
         <is>
           <t>This expert-level certification focuses on the front-end aspects of Adobe Commerce (Magento). It includes skills in front-end development, theme customization, and optimizing the user experience across devices.</t>
@@ -2897,17 +2612,17 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>Adobe Commerce (Magento), Front-End Development Tools</t>
+          <t>Adobe Commerce (Magento);Front-End Development Tools</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>Front-End Developer, UX/UI Designer, eCommerce Front-End Developer, Web Developer, Digital Designer</t>
+          <t>Front-End Developer;UX/UI Designer;eCommerce Front-End Developer;Web Developer;Digital Designer</t>
         </is>
       </c>
       <c r="J58" t="inlineStr">
         <is>
-          <t>Expert</t>
+          <t>EXPERT</t>
         </is>
       </c>
     </row>
@@ -2922,11 +2637,6 @@
           <t>CER-000058</t>
         </is>
       </c>
-      <c r="C59" t="inlineStr">
-        <is>
-          <t>Adobe</t>
-        </is>
-      </c>
       <c r="D59" t="inlineStr">
         <is>
           <t>This certification focuses on professional-level front-end development skills for Adobe Commerce. It covers responsive design, theme customization, and integration of third-party tools.</t>
@@ -2939,17 +2649,17 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>Adobe Commerce (Magento), Front-End Development Tools</t>
+          <t>Adobe Commerce (Magento);Front-End Development Tools</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>Front-End Developer, UX/UI Developer, Web Developer, eCommerce Developer, Digital Experience Designer</t>
+          <t>Front-End Developer;UX/UI Developer;Web Developer;eCommerce Developer;Digital Experience Designer</t>
         </is>
       </c>
       <c r="J59" t="inlineStr">
         <is>
-          <t>Advanced</t>
+          <t>ADVANCED</t>
         </is>
       </c>
     </row>
@@ -2964,11 +2674,6 @@
           <t>CER-000059</t>
         </is>
       </c>
-      <c r="C60" t="inlineStr">
-        <is>
-          <t>Adobe</t>
-        </is>
-      </c>
       <c r="D60" t="inlineStr">
         <is>
           <t>Validates ability to set up, manage, and host online meetings, webinars, and e-learning sessions using Adobe Connect Pro 7.</t>
@@ -2986,12 +2691,12 @@
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>Virtual Event Producer, LMS Administrator, Technical Trainer, Webinar Specialist, IT Support Engineer</t>
+          <t>Virtual Event Producer;LMS Administrator;Technical Trainer;Webinar Specialist;IT Support Engineer</t>
         </is>
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>Intermediate</t>
+          <t>INTERMEDIATE</t>
         </is>
       </c>
     </row>
@@ -3006,11 +2711,6 @@
           <t>CER-000060</t>
         </is>
       </c>
-      <c r="C61" t="inlineStr">
-        <is>
-          <t>Adobe</t>
-        </is>
-      </c>
       <c r="D61" t="inlineStr">
         <is>
           <t>This certification covers using Adobe Customer Journey Analytics to analyze customer data and optimize marketing strategies. It focuses on understanding and applying analytics to enhance customer journeys across channels.</t>
@@ -3023,17 +2723,17 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>Adobe Customer Journey Analytics, Customer Data Tools</t>
+          <t>Adobe Customer Journey Analytics;Customer Data Tools</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>Data Analyst, Marketing Analyst, Customer Experience Specialist, Digital Marketing Manager, Insights Analyst</t>
+          <t>Data Analyst;Marketing Analyst;Customer Experience Specialist;Digital Marketing Manager;Insights Analyst</t>
         </is>
       </c>
       <c r="J61" t="inlineStr">
         <is>
-          <t>Advanced</t>
+          <t>ADVANCED</t>
         </is>
       </c>
     </row>
@@ -3048,11 +2748,6 @@
           <t>CER-000061</t>
         </is>
       </c>
-      <c r="C62" t="inlineStr">
-        <is>
-          <t>Adobe</t>
-        </is>
-      </c>
       <c r="D62" t="inlineStr">
         <is>
           <t>This certification focuses on advanced technical skills required to integrate and customize Adobe Customer Journey Analytics. It covers data collection, implementation, and custom reporting to enhance customer experience strategies.</t>
@@ -3065,17 +2760,17 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>Adobe Customer Journey Analytics, Data Integration Tools</t>
+          <t>Adobe Customer Journey Analytics;Data Integration Tools</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>Data Integration Specialist, Marketing Data Developer, Analytics Developer, Digital Transformation Consultant, Data Engineer</t>
+          <t>Data Integration Specialist;Marketing Data Developer;Analytics Developer;Digital Transformation Consultant;Data Engineer</t>
         </is>
       </c>
       <c r="J62" t="inlineStr">
         <is>
-          <t>Expert</t>
+          <t>EXPERT</t>
         </is>
       </c>
     </row>
@@ -3090,11 +2785,6 @@
           <t>CER-000062</t>
         </is>
       </c>
-      <c r="C63" t="inlineStr">
-        <is>
-          <t>Adobe</t>
-        </is>
-      </c>
       <c r="D63" t="inlineStr">
         <is>
           <t>This certification covers the core development skills necessary to implement and configure Adobe Customer Journey Analytics. It includes building custom reports, integrating data sources, and analyzing customer journeys.</t>
@@ -3107,17 +2797,17 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>Adobe Customer Journey Analytics, Analytics Tools</t>
+          <t>Adobe Customer Journey Analytics;Analytics Tools</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>Analytics Developer, Data Integration Engineer, Customer Experience Developer, Marketing Analyst, Data Scientist</t>
+          <t>Analytics Developer;Data Integration Engineer;Customer Experience Developer;Marketing Analyst;Data Scientist</t>
         </is>
       </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>Advanced</t>
+          <t>ADVANCED</t>
         </is>
       </c>
     </row>
@@ -3132,11 +2822,6 @@
           <t>CER-000063</t>
         </is>
       </c>
-      <c r="C64" t="inlineStr">
-        <is>
-          <t>Adobe</t>
-        </is>
-      </c>
       <c r="D64" t="inlineStr">
         <is>
           <t>This certification is for professionals using Adobe Document Cloud to manage document workflows, digital signatures, and document collaboration. It emphasizes optimizing business processes and improving productivity.</t>
@@ -3149,17 +2834,17 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>Adobe Document Cloud, Document Workflow Tools</t>
+          <t>Adobe Document Cloud;Document Workflow Tools</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>Document Management Specialist, Workflow Consultant, IT Project Manager, Document Solutions Specialist, Business Process Analyst</t>
+          <t>Document Management Specialist;Workflow Consultant;IT Project Manager;Document Solutions Specialist;Business Process Analyst</t>
         </is>
       </c>
       <c r="J64" t="inlineStr">
         <is>
-          <t>Advanced</t>
+          <t>ADVANCED</t>
         </is>
       </c>
     </row>
@@ -3174,11 +2859,6 @@
           <t>CER-000064</t>
         </is>
       </c>
-      <c r="C65" t="inlineStr">
-        <is>
-          <t>Adobe</t>
-        </is>
-      </c>
       <c r="D65" t="inlineStr">
         <is>
           <t>Recognizes expertise in architecting scalable AEM solutions including infrastructure, integration, and customization.</t>
@@ -3196,12 +2876,12 @@
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>AEM Architect, Solutions Architect, Technical Lead, Systems Integrator, Web Platform Engineer</t>
+          <t>AEM Architect;Solutions Architect;Technical Lead;Systems Integrator;Web Platform Engineer</t>
         </is>
       </c>
       <c r="J65" t="inlineStr">
         <is>
-          <t>Expert</t>
+          <t>EXPERT</t>
         </is>
       </c>
     </row>
@@ -3216,11 +2896,6 @@
           <t>CER-000065</t>
         </is>
       </c>
-      <c r="C66" t="inlineStr">
-        <is>
-          <t>Adobe</t>
-        </is>
-      </c>
       <c r="D66" t="inlineStr">
         <is>
           <t>This certification focuses on migrating and optimizing Adobe Experience Manager (AEM) solutions to Adobe Experience Manager as a Cloud Service. It includes best practices for cloud architecture, data migration, and seamless transitions.</t>
@@ -3233,17 +2908,17 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>Adobe Experience Manager, Cloud Service Platforms</t>
+          <t>Adobe Experience Manager;Cloud Service Platforms</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>Cloud Architect, AEM Migration Specialist, Cloud Solutions Consultant, Systems Engineer, Digital Experience Architect</t>
+          <t>Cloud Architect;AEM Migration Specialist;Cloud Solutions Consultant;Systems Engineer;Digital Experience Architect</t>
         </is>
       </c>
       <c r="J66" t="inlineStr">
         <is>
-          <t>Expert</t>
+          <t>EXPERT</t>
         </is>
       </c>
     </row>
@@ -3258,11 +2933,6 @@
           <t>CER-000066</t>
         </is>
       </c>
-      <c r="C67" t="inlineStr">
-        <is>
-          <t>Adobe</t>
-        </is>
-      </c>
       <c r="D67" t="inlineStr">
         <is>
           <t>This certification covers advanced skills for managing and developing digital assets within Adobe Experience Manager. It includes creating and optimizing asset workflows, metadata management, and asset-driven marketing strategies.</t>
@@ -3275,17 +2945,17 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>Adobe Experience Manager, Digital Asset Management Tools</t>
+          <t>Adobe Experience Manager;Digital Asset Management Tools</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>AEM Assets Developer, Digital Asset Manager, Web Developer, Content Management Specialist, AEM Developer</t>
+          <t>AEM Assets Developer;Digital Asset Manager;Web Developer;Content Management Specialist;AEM Developer</t>
         </is>
       </c>
       <c r="J67" t="inlineStr">
         <is>
-          <t>Advanced</t>
+          <t>ADVANCED</t>
         </is>
       </c>
     </row>
@@ -3300,11 +2970,6 @@
           <t>CER-000067</t>
         </is>
       </c>
-      <c r="C68" t="inlineStr">
-        <is>
-          <t>Adobe</t>
-        </is>
-      </c>
       <c r="D68" t="inlineStr">
         <is>
           <t>This certification focuses on backend development skills for managing forms in Adobe Experience Manager. It includes creating dynamic forms, managing form data, and integrating them with enterprise systems.</t>
@@ -3317,17 +2982,17 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>Adobe Experience Manager, Backend Development Tools</t>
+          <t>Adobe Experience Manager;Backend Development Tools</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>AEM Backend Developer, Forms Developer, Web Developer, CMS Developer, Digital Experience Specialist</t>
+          <t>AEM Backend Developer;Forms Developer;Web Developer;CMS Developer;Digital Experience Specialist</t>
         </is>
       </c>
       <c r="J68" t="inlineStr">
         <is>
-          <t>Advanced</t>
+          <t>ADVANCED</t>
         </is>
       </c>
     </row>
@@ -3342,11 +3007,6 @@
           <t>CER-000068</t>
         </is>
       </c>
-      <c r="C69" t="inlineStr">
-        <is>
-          <t>Adobe</t>
-        </is>
-      </c>
       <c r="D69" t="inlineStr">
         <is>
           <t>This certification is designed for professionals focused on business processes within Adobe Experience Manager. It covers content management, site optimization, and user experience strategies in AEM.</t>
@@ -3359,17 +3019,17 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>Adobe Experience Manager, Content Management Tools</t>
+          <t>Adobe Experience Manager;Content Management Tools</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>Content Manager, Digital Experience Manager, Web Content Specialist, Marketing Manager, AEM Specialist</t>
+          <t>Content Manager;Digital Experience Manager;Web Content Specialist;Marketing Manager;AEM Specialist</t>
         </is>
       </c>
       <c r="J69" t="inlineStr">
         <is>
-          <t>Advanced</t>
+          <t>ADVANCED</t>
         </is>
       </c>
     </row>
@@ -3384,11 +3044,6 @@
           <t>CER-000069</t>
         </is>
       </c>
-      <c r="C70" t="inlineStr">
-        <is>
-          <t>Adobe</t>
-        </is>
-      </c>
       <c r="D70" t="inlineStr">
         <is>
           <t>Validates skills in building, configuring, and deploying AEM components, templates, and workflows.</t>
@@ -3406,12 +3061,12 @@
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>AEM Developer, Web Developer, CMS Engineer, Front-End Developer, Digital Experience Engineer</t>
+          <t>AEM Developer;Web Developer;CMS Engineer;Front-End Developer;Digital Experience Engineer</t>
         </is>
       </c>
       <c r="J70" t="inlineStr">
         <is>
-          <t>Intermediate</t>
+          <t>INTERMEDIATE</t>
         </is>
       </c>
     </row>
@@ -3426,11 +3081,6 @@
           <t>CER-000070</t>
         </is>
       </c>
-      <c r="C71" t="inlineStr">
-        <is>
-          <t>Adobe</t>
-        </is>
-      </c>
       <c r="D71" t="inlineStr">
         <is>
           <t>The DevOps Engineer Expert certification focuses on the deployment, maintenance, and scalability of Adobe Experience Manager solutions. It covers cloud configurations, continuous integration, and automated deployment processes.</t>
@@ -3443,17 +3093,17 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>Adobe Experience Manager, Cloud Infrastructure Tools</t>
+          <t>Adobe Experience Manager;Cloud Infrastructure Tools</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>DevOps Engineer, Cloud Infrastructure Engineer, AEM Operations Manager, Site Reliability Engineer, Systems Administrator</t>
+          <t>DevOps Engineer;Cloud Infrastructure Engineer;AEM Operations Manager;Site Reliability Engineer;Systems Administrator</t>
         </is>
       </c>
       <c r="J71" t="inlineStr">
         <is>
-          <t>Expert</t>
+          <t>EXPERT</t>
         </is>
       </c>
     </row>
@@ -3468,11 +3118,6 @@
           <t>CER-000071</t>
         </is>
       </c>
-      <c r="C72" t="inlineStr">
-        <is>
-          <t>Adobe</t>
-        </is>
-      </c>
       <c r="D72" t="inlineStr">
         <is>
           <t>This certification focuses on managing and organizing digital content within Adobe Experience Manager. It includes tasks such as content curation, metadata management, and content accessibility strategies.</t>
@@ -3485,17 +3130,17 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>Adobe Experience Manager, Digital Content Management</t>
+          <t>Adobe Experience Manager;Digital Content Management</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>Digital Librarian, Content Manager, Web Content Specialist, Digital Archivist, AEM Content Specialist</t>
+          <t>Digital Librarian;Content Manager;Web Content Specialist;Digital Archivist;AEM Content Specialist</t>
         </is>
       </c>
       <c r="J72" t="inlineStr">
         <is>
-          <t>Advanced</t>
+          <t>ADVANCED</t>
         </is>
       </c>
     </row>
@@ -3510,11 +3155,6 @@
           <t>CER-000072</t>
         </is>
       </c>
-      <c r="C73" t="inlineStr">
-        <is>
-          <t>Adobe</t>
-        </is>
-      </c>
       <c r="D73" t="inlineStr">
         <is>
           <t>This certification is for advanced developers specializing in the creation and customization of dynamic forms within Adobe Experience Manager (AEM). It focuses on integrating complex form workflows, data collection, and enterprise system connections.</t>
@@ -3527,17 +3167,17 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>Adobe Experience Manager, AEM Forms</t>
+          <t>Adobe Experience Manager;AEM Forms</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>AEM Forms Developer, Web Developer, CMS Developer, Digital Experience Developer, Forms Specialist</t>
+          <t>AEM Forms Developer;Web Developer;CMS Developer;Digital Experience Developer;Forms Specialist</t>
         </is>
       </c>
       <c r="J73" t="inlineStr">
         <is>
-          <t>Expert</t>
+          <t>EXPERT</t>
         </is>
       </c>
     </row>
@@ -3552,11 +3192,6 @@
           <t>CER-000073</t>
         </is>
       </c>
-      <c r="C74" t="inlineStr">
-        <is>
-          <t>Adobe</t>
-        </is>
-      </c>
       <c r="D74" t="inlineStr">
         <is>
           <t>This master-level certification focuses on AEM Sites architecture. It covers advanced topics such as site architecture design, scalability, cloud deployment, and integration with third-party systems. It is ideal for those looking to lead AEM Sites implementations.</t>
@@ -3569,17 +3204,17 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>Adobe Experience Manager, AEM Sites</t>
+          <t>Adobe Experience Manager;AEM Sites</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>AEM Solutions Architect, Site Architect, Digital Experience Architect, Technical Lead, CMS Architect</t>
+          <t>AEM Solutions Architect;Site Architect;Digital Experience Architect;Technical Lead;CMS Architect</t>
         </is>
       </c>
       <c r="J74" t="inlineStr">
         <is>
-          <t>Expert</t>
+          <t>EXPERT</t>
         </is>
       </c>
     </row>
@@ -3594,11 +3229,6 @@
           <t>CER-000074</t>
         </is>
       </c>
-      <c r="C75" t="inlineStr">
-        <is>
-          <t>Adobe</t>
-        </is>
-      </c>
       <c r="D75" t="inlineStr">
         <is>
           <t>This certification focuses on using Adobe Experience Manager Sites to create and optimize customer-facing websites and digital content. It includes content management, site optimization, and the effective use of AEM for web content management.</t>
@@ -3611,17 +3241,17 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>Adobe Experience Manager, Web Content Management Tools</t>
+          <t>Adobe Experience Manager;Web Content Management Tools</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>Digital Content Manager, Marketing Manager, Content Strategist, AEM Site Specialist, Business Analyst</t>
+          <t>Digital Content Manager;Marketing Manager;Content Strategist;AEM Site Specialist;Business Analyst</t>
         </is>
       </c>
       <c r="J75" t="inlineStr">
         <is>
-          <t>Expert</t>
+          <t>EXPERT</t>
         </is>
       </c>
     </row>
@@ -3636,11 +3266,6 @@
           <t>CER-000075</t>
         </is>
       </c>
-      <c r="C76" t="inlineStr">
-        <is>
-          <t>Adobe</t>
-        </is>
-      </c>
       <c r="D76" t="inlineStr">
         <is>
           <t>This certification is aimed at professionals who manage content creation and publishing within AEM Sites. It covers content authoring, content governance, and basic site management strategies in AEM.</t>
@@ -3653,17 +3278,17 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>Adobe Experience Manager, Content Management Tools</t>
+          <t>Adobe Experience Manager;Content Management Tools</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>Content Author, Web Content Specialist, Digital Marketing Specialist, AEM Content Manager, Content Strategist</t>
+          <t>Content Author;Web Content Specialist;Digital Marketing Specialist;AEM Content Manager;Content Strategist</t>
         </is>
       </c>
       <c r="J76" t="inlineStr">
         <is>
-          <t>Advanced</t>
+          <t>ADVANCED</t>
         </is>
       </c>
     </row>
@@ -3678,11 +3303,6 @@
           <t>CER-000076</t>
         </is>
       </c>
-      <c r="C77" t="inlineStr">
-        <is>
-          <t>Adobe</t>
-        </is>
-      </c>
       <c r="D77" t="inlineStr">
         <is>
           <t>This expert-level certification focuses on advanced development skills for AEM Sites. It includes component development, integration, and customizations for optimizing website performance, scalability, and user experience.</t>
@@ -3695,17 +3315,17 @@
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>Adobe Experience Manager, AEM Sites Development</t>
+          <t>Adobe Experience Manager;AEM Sites Development</t>
         </is>
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>AEM Developer, Web Developer, Full-Stack Developer, AEM Solutions Developer, Site Developer</t>
+          <t>AEM Developer;Web Developer;Full-Stack Developer;AEM Solutions Developer;Site Developer</t>
         </is>
       </c>
       <c r="J77" t="inlineStr">
         <is>
-          <t>Expert</t>
+          <t>EXPERT</t>
         </is>
       </c>
     </row>
@@ -3720,11 +3340,6 @@
           <t>CER-000077</t>
         </is>
       </c>
-      <c r="C78" t="inlineStr">
-        <is>
-          <t>Adobe</t>
-        </is>
-      </c>
       <c r="D78" t="inlineStr">
         <is>
           <t>This certification covers key development skills needed for AEM Sites. It focuses on creating and customizing components, templates, and pages to optimize site performance and meet business requirements.</t>
@@ -3737,17 +3352,17 @@
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>Adobe Experience Manager, Web Development Tools</t>
+          <t>Adobe Experience Manager;Web Development Tools</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>AEM Developer, Web Developer, Front-End Developer, Full-Stack Developer, CMS Developer</t>
+          <t>AEM Developer;Web Developer;Front-End Developer;Full-Stack Developer;CMS Developer</t>
         </is>
       </c>
       <c r="J78" t="inlineStr">
         <is>
-          <t>Advanced</t>
+          <t>ADVANCED</t>
         </is>
       </c>
     </row>
@@ -3762,11 +3377,6 @@
           <t>CER-000078</t>
         </is>
       </c>
-      <c r="C79" t="inlineStr">
-        <is>
-          <t>Adobe</t>
-        </is>
-      </c>
       <c r="D79" t="inlineStr">
         <is>
           <t>This certification provides foundational knowledge of Adobe Experience Manager, including core concepts such as content management, workflows, and site architecture. It is ideal for individuals new to AEM.</t>
@@ -3779,17 +3389,17 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>Adobe Experience Manager, CMS Tools</t>
+          <t>Adobe Experience Manager;CMS Tools</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>AEM Developer, CMS Developer, Digital Marketing Specialist, Web Developer, Technical Consultant</t>
+          <t>AEM Developer;CMS Developer;Digital Marketing Specialist;Web Developer;Technical Consultant</t>
         </is>
       </c>
       <c r="J79" t="inlineStr">
         <is>
-          <t>Advanced</t>
+          <t>ADVANCED</t>
         </is>
       </c>
     </row>
@@ -3804,11 +3414,6 @@
           <t>CER-000079</t>
         </is>
       </c>
-      <c r="C80" t="inlineStr">
-        <is>
-          <t>Adobe</t>
-        </is>
-      </c>
       <c r="D80" t="inlineStr">
         <is>
           <t>This is a beta certification focused on Adobe Firefly, Adobe's generative AI platform. It covers the basics of using Firefly for content creation, AI-driven marketing, and automating workflows with Adobe tools.</t>
@@ -3821,17 +3426,17 @@
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>Adobe Firefly, AI Tools</t>
+          <t>Adobe Firefly;AI Tools</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>Digital Content Creator, AI Specialist, Marketing Specialist, Automation Expert, Data Scientist</t>
+          <t>Digital Content Creator;AI Specialist;Marketing Specialist;Automation Expert;Data Scientist</t>
         </is>
       </c>
       <c r="J80" t="inlineStr">
         <is>
-          <t>Beginner</t>
+          <t>BEGINNER</t>
         </is>
       </c>
     </row>
@@ -3846,11 +3451,6 @@
           <t>CER-000080</t>
         </is>
       </c>
-      <c r="C81" t="inlineStr">
-        <is>
-          <t>Adobe</t>
-        </is>
-      </c>
       <c r="D81" t="inlineStr">
         <is>
           <t>This certification focuses on the use of Adobe Journey Optimizer for orchestrating personalized customer journeys. It covers strategies for optimizing marketing workflows and improving customer engagement across channels.</t>
@@ -3863,17 +3463,17 @@
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>Adobe Journey Optimizer, Marketing Automation Tools</t>
+          <t>Adobe Journey Optimizer;Marketing Automation Tools</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>Marketing Manager, Campaign Manager, Customer Journey Specialist, Digital Marketing Analyst, Customer Experience Manager</t>
+          <t>Marketing Manager;Campaign Manager;Customer Journey Specialist;Digital Marketing Analyst;Customer Experience Manager</t>
         </is>
       </c>
       <c r="J81" t="inlineStr">
         <is>
-          <t>Advanced</t>
+          <t>ADVANCED</t>
         </is>
       </c>
     </row>
@@ -3888,11 +3488,6 @@
           <t>CER-000081</t>
         </is>
       </c>
-      <c r="C82" t="inlineStr">
-        <is>
-          <t>Adobe</t>
-        </is>
-      </c>
       <c r="D82" t="inlineStr">
         <is>
           <t>This expert-level certification is for developers working with Adobe Journey Optimizer. It focuses on advanced customization, integrations, and implementing AI-powered personalization techniques to optimize customer journeys.</t>
@@ -3905,17 +3500,17 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>Adobe Journey Optimizer, Marketing Automation Development</t>
+          <t>Adobe Journey Optimizer;Marketing Automation Development</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>Journey Optimizer Developer, Marketing Automation Developer, Full-Stack Developer, Technical Consultant, Digital Experience Developer</t>
+          <t>Journey Optimizer Developer;Marketing Automation Developer;Full-Stack Developer;Technical Consultant;Digital Experience Developer</t>
         </is>
       </c>
       <c r="J82" t="inlineStr">
         <is>
-          <t>Expert</t>
+          <t>EXPERT</t>
         </is>
       </c>
     </row>
@@ -3930,11 +3525,6 @@
           <t>CER-000082</t>
         </is>
       </c>
-      <c r="C83" t="inlineStr">
-        <is>
-          <t>Adobe</t>
-        </is>
-      </c>
       <c r="D83" t="inlineStr">
         <is>
           <t>This master-level certification is for architects designing and deploying marketing solutions using Adobe Marketo Engage. It focuses on advanced Marketo implementations, integration with other platforms, and optimizing marketing workflows at scale.</t>
@@ -3947,17 +3537,17 @@
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>Adobe Marketo Engage, Marketing Automation Solutions</t>
+          <t>Adobe Marketo Engage;Marketing Automation Solutions</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>Marketing Solutions Architect, Marketing Automation Architect, Senior Marketing Consultant, Digital Marketing Strategist, Marketing Technology Specialist</t>
+          <t>Marketing Solutions Architect;Marketing Automation Architect;Senior Marketing Consultant;Digital Marketing Strategist;Marketing Technology Specialist</t>
         </is>
       </c>
       <c r="J83" t="inlineStr">
         <is>
-          <t>Expert</t>
+          <t>EXPERT</t>
         </is>
       </c>
     </row>
@@ -3972,11 +3562,6 @@
           <t>CER-000083</t>
         </is>
       </c>
-      <c r="C84" t="inlineStr">
-        <is>
-          <t>Adobe</t>
-        </is>
-      </c>
       <c r="D84" t="inlineStr">
         <is>
           <t>This certification focuses on mastering business strategies within Adobe Marketo Engage, including campaign creation, lead management, and measuring marketing effectiveness through analytics.</t>
@@ -3989,17 +3574,17 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>Adobe Marketo Engage, Marketing Automation Tools</t>
+          <t>Adobe Marketo Engage;Marketing Automation Tools</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>Marketing Manager, Campaign Manager, Marketing Analyst, Lead Generation Specialist, Digital Marketing Strategist</t>
+          <t>Marketing Manager;Campaign Manager;Marketing Analyst;Lead Generation Specialist;Digital Marketing Strategist</t>
         </is>
       </c>
       <c r="J84" t="inlineStr">
         <is>
-          <t>Expert</t>
+          <t>EXPERT</t>
         </is>
       </c>
     </row>
@@ -4014,11 +3599,6 @@
           <t>CER-000084</t>
         </is>
       </c>
-      <c r="C85" t="inlineStr">
-        <is>
-          <t>Adobe</t>
-        </is>
-      </c>
       <c r="D85" t="inlineStr">
         <is>
           <t>This certification focuses on practical application of Adobe Marketo Engage for campaign management, lead nurturing, and marketing automation at an operational level.</t>
@@ -4031,17 +3611,17 @@
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>Adobe Marketo Engage, Marketing Automation Tools</t>
+          <t>Adobe Marketo Engage;Marketing Automation Tools</t>
         </is>
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>Marketing Specialist, Campaign Manager, Digital Marketing Specialist, Marketing Operations Manager, Lead Generation Expert</t>
+          <t>Marketing Specialist;Campaign Manager;Digital Marketing Specialist;Marketing Operations Manager;Lead Generation Expert</t>
         </is>
       </c>
       <c r="J85" t="inlineStr">
         <is>
-          <t>Advanced</t>
+          <t>ADVANCED</t>
         </is>
       </c>
     </row>
@@ -4056,11 +3636,6 @@
           <t>CER-000085</t>
         </is>
       </c>
-      <c r="C86" t="inlineStr">
-        <is>
-          <t>Adobe</t>
-        </is>
-      </c>
       <c r="D86" t="inlineStr">
         <is>
           <t>This certification is aimed at digital marketers using Adobe Marketo Engage for creating and optimizing digital campaigns. It covers email marketing, lead nurturing, and engagement strategies.</t>
@@ -4073,17 +3648,17 @@
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>Adobe Marketo Engage, Digital Marketing Tools</t>
+          <t>Adobe Marketo Engage;Digital Marketing Tools</t>
         </is>
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>Digital Marketing Manager, Email Marketing Specialist, Campaign Manager, Content Marketing Specialist, Digital Campaign Strategist</t>
+          <t>Digital Marketing Manager;Email Marketing Specialist;Campaign Manager;Content Marketing Specialist;Digital Campaign Strategist</t>
         </is>
       </c>
       <c r="J86" t="inlineStr">
         <is>
-          <t>Advanced</t>
+          <t>ADVANCED</t>
         </is>
       </c>
     </row>
@@ -4098,11 +3673,6 @@
           <t>CER-000086</t>
         </is>
       </c>
-      <c r="C87" t="inlineStr">
-        <is>
-          <t>Adobe</t>
-        </is>
-      </c>
       <c r="D87" t="inlineStr">
         <is>
           <t>This is the Japanese-language version of the Adobe Marketo Engage Professional certification. It focuses on marketing automation tools and strategies for professionals in Japan, covering campaign management and optimization.</t>
@@ -4115,17 +3685,17 @@
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>Adobe Marketo Engage, Marketing Automation Tools</t>
+          <t>Adobe Marketo Engage;Marketing Automation Tools</t>
         </is>
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>Digital Marketing Manager, Campaign Specialist, Marketing Operations Manager, Marketing Automation Specialist, Lead Nurturing Expert</t>
+          <t>Digital Marketing Manager;Campaign Specialist;Marketing Operations Manager;Marketing Automation Specialist;Lead Nurturing Expert</t>
         </is>
       </c>
       <c r="J87" t="inlineStr">
         <is>
-          <t>Advanced</t>
+          <t>ADVANCED</t>
         </is>
       </c>
     </row>
@@ -4140,11 +3710,6 @@
           <t>CER-000087</t>
         </is>
       </c>
-      <c r="C88" t="inlineStr">
-        <is>
-          <t>Adobe</t>
-        </is>
-      </c>
       <c r="D88" t="inlineStr">
         <is>
           <t>This certification covers the use of Adobe Real-Time Customer Data Platform (CDP) to unify customer data and personalize marketing campaigns. It focuses on customer segmentation, journey mapping, and real-time insights for optimized marketing.</t>
@@ -4157,17 +3722,17 @@
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>Adobe Real-Time CDP, Customer Data Platforms</t>
+          <t>Adobe Real-Time CDP;Customer Data Platforms</t>
         </is>
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>Data Analyst, Campaign Manager, Customer Insights Manager, Marketing Automation Specialist, Digital Experience Manager</t>
+          <t>Data Analyst;Campaign Manager;Customer Insights Manager;Marketing Automation Specialist;Digital Experience Manager</t>
         </is>
       </c>
       <c r="J88" t="inlineStr">
         <is>
-          <t>Advanced</t>
+          <t>ADVANCED</t>
         </is>
       </c>
     </row>
@@ -4182,11 +3747,6 @@
           <t>CER-000088</t>
         </is>
       </c>
-      <c r="C89" t="inlineStr">
-        <is>
-          <t>Adobe</t>
-        </is>
-      </c>
       <c r="D89" t="inlineStr">
         <is>
           <t>This expert-level certification focuses on developing and customizing Adobe Real-Time Customer Data Platform (CDP) solutions. It covers data integration, custom event tracking, and advanced customer segmentation to optimize real-time marketing efforts.</t>
@@ -4199,17 +3759,17 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>Adobe Real-Time CDP, Data Integration Tools</t>
+          <t>Adobe Real-Time CDP;Data Integration Tools</t>
         </is>
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>CDP Developer, Data Integration Specialist, Marketing Solutions Architect, Real-Time Marketing Specialist, Customer Data Engineer</t>
+          <t>CDP Developer;Data Integration Specialist;Marketing Solutions Architect;Real-Time Marketing Specialist;Customer Data Engineer</t>
         </is>
       </c>
       <c r="J89" t="inlineStr">
         <is>
-          <t>Expert</t>
+          <t>EXPERT</t>
         </is>
       </c>
     </row>
@@ -4224,11 +3784,6 @@
           <t>CER-000089</t>
         </is>
       </c>
-      <c r="C90" t="inlineStr">
-        <is>
-          <t>Adobe</t>
-        </is>
-      </c>
       <c r="D90" t="inlineStr">
         <is>
           <t>This master-level certification focuses on architecting Adobe Target solutions to drive personalized customer experiences. It includes advanced topics such as targeting strategies, A/B testing, integration with other Adobe solutions, and optimization techniques.</t>
@@ -4241,17 +3796,17 @@
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>Adobe Target, Personalization Tools</t>
+          <t>Adobe Target;Personalization Tools</t>
         </is>
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>Marketing Architect, Personalization Architect, Digital Experience Architect, Optimization Specialist, Data Solutions Architect</t>
+          <t>Marketing Architect;Personalization Architect;Digital Experience Architect;Optimization Specialist;Data Solutions Architect</t>
         </is>
       </c>
       <c r="J90" t="inlineStr">
         <is>
-          <t>Expert</t>
+          <t>EXPERT</t>
         </is>
       </c>
     </row>
@@ -4266,11 +3821,6 @@
           <t>CER-000090</t>
         </is>
       </c>
-      <c r="C91" t="inlineStr">
-        <is>
-          <t>Adobe</t>
-        </is>
-      </c>
       <c r="D91" t="inlineStr">
         <is>
           <t>This certification is for professionals who have mastered business strategies within Adobe Target. It covers campaign management, personalization, A/B testing, and analyzing optimization results for improving customer engagement.</t>
@@ -4283,17 +3833,17 @@
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>Adobe Target, Marketing Optimization Tools</t>
+          <t>Adobe Target;Marketing Optimization Tools</t>
         </is>
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>Digital Marketing Manager, Personalization Expert, Campaign Manager, Optimization Specialist, Customer Experience Manager</t>
+          <t>Digital Marketing Manager;Personalization Expert;Campaign Manager;Optimization Specialist;Customer Experience Manager</t>
         </is>
       </c>
       <c r="J91" t="inlineStr">
         <is>
-          <t>Expert</t>
+          <t>EXPERT</t>
         </is>
       </c>
     </row>
@@ -4308,11 +3858,6 @@
           <t>CER-000091</t>
         </is>
       </c>
-      <c r="C92" t="inlineStr">
-        <is>
-          <t>Adobe</t>
-        </is>
-      </c>
       <c r="D92" t="inlineStr">
         <is>
           <t>This certification focuses on applying Adobe Target's personalization and optimization features in marketing campaigns. It covers A/B testing, targeting strategies, and performance analysis to enhance customer experiences.</t>
@@ -4325,17 +3870,17 @@
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>Adobe Target, Personalization Tools</t>
+          <t>Adobe Target;Personalization Tools</t>
         </is>
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>Campaign Manager, Personalization Specialist, Optimization Analyst, Digital Marketing Specialist, Marketing Operations Manager</t>
+          <t>Campaign Manager;Personalization Specialist;Optimization Analyst;Digital Marketing Specialist;Marketing Operations Manager</t>
         </is>
       </c>
       <c r="J92" t="inlineStr">
         <is>
-          <t>Advanced</t>
+          <t>ADVANCED</t>
         </is>
       </c>
     </row>
@@ -4350,11 +3895,6 @@
           <t>CER-000092</t>
         </is>
       </c>
-      <c r="C93" t="inlineStr">
-        <is>
-          <t>Adobe</t>
-        </is>
-      </c>
       <c r="D93" t="inlineStr">
         <is>
           <t>This certification is for professionals specializing in optimizing marketing campaigns using Adobe Target. It covers techniques for A/B testing, targeting, and audience segmentation to boost conversions and engagement.</t>
@@ -4367,17 +3907,17 @@
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>Adobe Target, Marketing Optimization Tools</t>
+          <t>Adobe Target;Marketing Optimization Tools</t>
         </is>
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>Optimization Specialist, A/B Testing Expert, Campaign Analyst, Marketing Automation Specialist, Digital Marketing Specialist</t>
+          <t>Optimization Specialist;A/B Testing Expert;Campaign Analyst;Marketing Automation Specialist;Digital Marketing Specialist</t>
         </is>
       </c>
       <c r="J93" t="inlineStr">
         <is>
-          <t>Advanced</t>
+          <t>ADVANCED</t>
         </is>
       </c>
     </row>
@@ -4392,11 +3932,6 @@
           <t>CER-000093</t>
         </is>
       </c>
-      <c r="C94" t="inlineStr">
-        <is>
-          <t>Adobe</t>
-        </is>
-      </c>
       <c r="D94" t="inlineStr">
         <is>
           <t>This certification is designed for developers working with Adobe Workfront. It covers advanced features such as custom integrations, API management, and automating workflows to optimize project management processes.</t>
@@ -4409,17 +3944,17 @@
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>Adobe Workfront, Project Management Tools</t>
+          <t>Adobe Workfront;Project Management Tools</t>
         </is>
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>Workfront Developer, Project Automation Specialist, Software Developer, API Integrations Engineer, Solutions Architect</t>
+          <t>Workfront Developer;Project Automation Specialist;Software Developer;API Integrations Engineer;Solutions Architect</t>
         </is>
       </c>
       <c r="J94" t="inlineStr">
         <is>
-          <t>Expert</t>
+          <t>EXPERT</t>
         </is>
       </c>
     </row>
@@ -4434,11 +3969,6 @@
           <t>CER-000094</t>
         </is>
       </c>
-      <c r="C95" t="inlineStr">
-        <is>
-          <t>Adobe</t>
-        </is>
-      </c>
       <c r="D95" t="inlineStr">
         <is>
           <t>This certification focuses on practical skills for developing and customizing Adobe Workfront solutions. It covers tasks like API integration, creating custom workflows, and managing tasks within the Workfront platform.</t>
@@ -4451,17 +3981,17 @@
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>Adobe Workfront, Project Management Tools</t>
+          <t>Adobe Workfront;Project Management Tools</t>
         </is>
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t>Workfront Developer, Project Management Specialist, Workflow Automation Developer, Web Developer, API Specialist</t>
+          <t>Workfront Developer;Project Management Specialist;Workflow Automation Developer;Web Developer;API Specialist</t>
         </is>
       </c>
       <c r="J95" t="inlineStr">
         <is>
-          <t>Advanced</t>
+          <t>ADVANCED</t>
         </is>
       </c>
     </row>
@@ -4476,11 +4006,6 @@
           <t>CER-000095</t>
         </is>
       </c>
-      <c r="C96" t="inlineStr">
-        <is>
-          <t>Adobe</t>
-        </is>
-      </c>
       <c r="D96" t="inlineStr">
         <is>
           <t>This expert certification covers integrating Adobe Workfront with Adobe Experience Manager (AEM). It focuses on advanced customization and automating project workflows between Workfront and AEM to enhance content management processes.</t>
@@ -4493,17 +4018,17 @@
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>Adobe Workfront, Adobe Experience Manager, Integration Tools</t>
+          <t>Adobe Workfront;Adobe Experience Manager;Integration Tools</t>
         </is>
       </c>
       <c r="H96" t="inlineStr">
         <is>
-          <t>AEM Integrations Specialist, Workfront Integration Engineer, Digital Project Manager, Workflow Automation Specialist, Content Operations Manager</t>
+          <t>AEM Integrations Specialist;Workfront Integration Engineer;Digital Project Manager;Workflow Automation Specialist;Content Operations Manager</t>
         </is>
       </c>
       <c r="J96" t="inlineStr">
         <is>
-          <t>Expert</t>
+          <t>EXPERT</t>
         </is>
       </c>
     </row>
@@ -4518,11 +4043,6 @@
           <t>CER-000096</t>
         </is>
       </c>
-      <c r="C97" t="inlineStr">
-        <is>
-          <t>Adobe</t>
-        </is>
-      </c>
       <c r="D97" t="inlineStr">
         <is>
           <t>This certification is for developers working with Adobe Workfront Fusion, focusing on building integrations and automating workflows across multiple platforms to improve project management and team collaboration.</t>
@@ -4535,17 +4055,17 @@
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>Adobe Workfront, Workflow Automation Tools</t>
+          <t>Adobe Workfront;Workflow Automation Tools</t>
         </is>
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>Workfront Fusion Developer, Integration Specialist, Automation Engineer, Software Developer, Technical Consultant</t>
+          <t>Workfront Fusion Developer;Integration Specialist;Automation Engineer;Software Developer;Technical Consultant</t>
         </is>
       </c>
       <c r="J97" t="inlineStr">
         <is>
-          <t>Advanced</t>
+          <t>ADVANCED</t>
         </is>
       </c>
     </row>
@@ -4560,11 +4080,6 @@
           <t>CER-000097</t>
         </is>
       </c>
-      <c r="C98" t="inlineStr">
-        <is>
-          <t>Adobe</t>
-        </is>
-      </c>
       <c r="D98" t="inlineStr">
         <is>
           <t>This is a beta-level certification for developers new to Adobe Workfront Fusion. It focuses on basic integration and workflow automation skills to streamline project management processes using Workfront Fusion.</t>
@@ -4577,17 +4092,17 @@
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>Adobe Workfront, Workflow Automation Tools</t>
+          <t>Adobe Workfront;Workflow Automation Tools</t>
         </is>
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>Integration Developer, Workfront Specialist, Automation Engineer, Project Management Assistant, Technical Support Specialist</t>
+          <t>Integration Developer;Workfront Specialist;Automation Engineer;Project Management Assistant;Technical Support Specialist</t>
         </is>
       </c>
       <c r="J98" t="inlineStr">
         <is>
-          <t>Beginner</t>
+          <t>BEGINNER</t>
         </is>
       </c>
     </row>
@@ -4602,11 +4117,6 @@
           <t>CER-000098</t>
         </is>
       </c>
-      <c r="C99" t="inlineStr">
-        <is>
-          <t>Adobe</t>
-        </is>
-      </c>
       <c r="D99" t="inlineStr">
         <is>
           <t>This certification focuses on managing projects efficiently using Adobe Workfront. It includes topics like resource allocation, project timelines, team collaboration, and optimizing project workflows for large-scale teams.</t>
@@ -4619,17 +4129,17 @@
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>Adobe Workfront, Project Management Tools</t>
+          <t>Adobe Workfront;Project Management Tools</t>
         </is>
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>Project Manager, Program Manager, Digital Project Manager, Project Coordinator, Operations Manager</t>
+          <t>Project Manager;Program Manager;Digital Project Manager;Project Coordinator;Operations Manager</t>
         </is>
       </c>
       <c r="J99" t="inlineStr">
         <is>
-          <t>Advanced</t>
+          <t>ADVANCED</t>
         </is>
       </c>
     </row>
@@ -4644,11 +4154,6 @@
           <t>CER-000099</t>
         </is>
       </c>
-      <c r="C100" t="inlineStr">
-        <is>
-          <t>Adobe (Magento)</t>
-        </is>
-      </c>
       <c r="D100" t="inlineStr">
         <is>
           <t>Demonstrates understanding of Magento 2 architecture, customization, and module development.</t>
@@ -4666,12 +4171,12 @@
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>Web Developer, eCommerce Developer, PHP Engineer</t>
+          <t>Web Developer;eCommerce Developer;PHP Engineer</t>
         </is>
       </c>
       <c r="J100" t="inlineStr">
         <is>
-          <t>Intermediate</t>
+          <t>INTERMEDIATE</t>
         </is>
       </c>
     </row>
@@ -4686,11 +4191,6 @@
           <t>CER-000100</t>
         </is>
       </c>
-      <c r="C101" t="inlineStr">
-        <is>
-          <t>Adobe (Magento)</t>
-        </is>
-      </c>
       <c r="D101" t="inlineStr">
         <is>
           <t>Focuses on developing, deploying, and maintaining Magento Commerce Cloud environments.</t>
@@ -4708,12 +4208,12 @@
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>Cloud Developer, eCommerce Specialist, DevOps Engineer</t>
+          <t>Cloud Developer;eCommerce Specialist;DevOps Engineer</t>
         </is>
       </c>
       <c r="J101" t="inlineStr">
         <is>
-          <t>Advanced</t>
+          <t>ADVANCED</t>
         </is>
       </c>
     </row>

</xml_diff>